<commit_message>
Korp Filial 07/2026: reembolso do Suporte mantido em 2891
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-07/Integracao_Dominio_Korp_Filial_07-2026.xlsx
+++ b/Korp/Filial/2026-07/Integracao_Dominio_Korp_Filial_07-2026.xlsx
@@ -46,7 +46,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,9 +114,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -493,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1540,7 +1532,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>85.75</v>
+        <v>1422.19</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
@@ -1549,42 +1541,42 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>617 - REEMBOLSO</t>
+          <t>8783 - DIAS FERIAS</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Folha</t>
+          <t>Férias</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>2891</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+          <t>2524</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>3152</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2524</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Lançado na Folha Pgto do Suporte; o plano só tem Reembolsos de Viagem no DES (3134)</t>
+          <t>Férias da Fernanda (gozo em 08/2026, pagas em 31/07) lançadas no ADM</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr"/>
@@ -1592,7 +1584,7 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>1422.19</v>
+        <v>475.37</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
@@ -1601,7 +1593,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>8783 - DIAS FERIAS</t>
+          <t>931 - 1/3 DAS FERIAS</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1636,7 +1628,7 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>Férias da Fernanda (gozo em 08/2026, pagas em 31/07) lançadas no ADM</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="K25" s="8" t="inlineStr"/>
@@ -1644,7 +1636,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>475.37</v>
+        <v>1.63</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
@@ -1653,7 +1645,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>931 - 1/3 DAS FERIAS</t>
+          <t>805 - MEDIA VALOR FERIAS</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1696,7 +1688,7 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>1.63</v>
+        <v>2.3</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
@@ -1705,7 +1697,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>805 - MEDIA VALOR FERIAS</t>
+          <t>806 - MEDIA HORAS FERIAS</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -1748,7 +1740,7 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>2.3</v>
+        <v>146.81</v>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
@@ -1757,7 +1749,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>806 - MEDIA HORAS FERIAS</t>
+          <t>812 - INSS FERIAS</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1767,22 +1759,22 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
+          <t>2524</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
           <t>3017</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>2524</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>3152</t>
-        </is>
-      </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>2524</t>
+          <t>2531</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -1792,7 +1784,7 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Idem</t>
+          <t>INSS das férias creditado em despesa</t>
         </is>
       </c>
       <c r="K28" s="8" t="inlineStr"/>
@@ -1800,41 +1792,41 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>146.81</v>
+        <v>497.96</v>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>8 - SD SUPORTE</t>
+          <t>9 - CONSULTORIA INTERNA E GP</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>812 - INSS FERIAS</t>
+          <t>302 - HORAS EXTRAS 75%</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Férias</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>2524</t>
+          <t>2577</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>2524</t>
+          <t>3151</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>2531</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -1842,17 +1834,13 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>INSS das férias creditado em despesa</t>
-        </is>
-      </c>
+      <c r="J29" s="7" t="inlineStr"/>
       <c r="K29" s="8" t="inlineStr"/>
       <c r="L29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>497.96</v>
+        <v>73.77</v>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
@@ -1861,7 +1849,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>302 - HORAS EXTRAS 75%</t>
+          <t>250 - REFLEXO EXTRAS DSR</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1900,7 +1888,7 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>73.77</v>
+        <v>35</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
@@ -1909,7 +1897,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>250 - REFLEXO EXTRAS DSR</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1919,22 +1907,22 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>2577</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>3148</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>3151</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2911</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -1948,55 +1936,59 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>35</v>
+        <v>650</v>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>9 - CONSULTORIA INTERNA E GP</t>
+          <t>10 - ADM FINANCEIRO</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
+          <t>8490 - BOLSA AUXILIO FERIAS</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Folha</t>
+          <t>Rescisão</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>3148</t>
+          <t>2524</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2995</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>2911</t>
+          <t>2526</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J32" s="7" t="inlineStr"/>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>Rescisão de estágio da Julia (23/07): bolsa de estagiário vai para Estagiários / Estágios a pagar</t>
+        </is>
+      </c>
       <c r="K32" s="8" t="inlineStr"/>
       <c r="L32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>650</v>
+        <v>216.67</v>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
@@ -2005,7 +1997,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>8490 - BOLSA AUXILIO FERIAS</t>
+          <t>8496 - BOLSA AUXILIO 1/3 FERIAS</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2040,7 +2032,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de estágio da Julia (23/07): bolsa de estagiário vai para Estagiários / Estágios a pagar</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr"/>
@@ -2048,7 +2040,7 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>216.67</v>
+        <v>325</v>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
@@ -2057,7 +2049,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>8496 - BOLSA AUXILIO 1/3 FERIAS</t>
+          <t>8490 - BOLSA AUXILIO FERIAS</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2067,12 +2059,12 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>2524</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2092,7 +2084,7 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Idem</t>
+          <t>Rescisão de estágio da Isabele (31/07) não saiu no TXT de 07; deve vir no TXT de 08 (como o Antônio)</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr"/>
@@ -2100,7 +2092,7 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>325</v>
+        <v>108.33</v>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
@@ -2109,7 +2101,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>8490 - BOLSA AUXILIO FERIAS</t>
+          <t>8496 - BOLSA AUXILIO 1/3 FERIAS</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2144,7 +2136,7 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de estágio da Isabele (31/07) não saiu no TXT de 07; deve vir no TXT de 08 (como o Antônio)</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="K35" s="8" t="inlineStr"/>
@@ -2152,7 +2144,7 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>108.33</v>
+        <v>1300</v>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
@@ -2161,7 +2153,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>8496 - BOLSA AUXILIO 1/3 FERIAS</t>
+          <t>8797 - DIAS BOLSA AUXILIO</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -2204,11 +2196,11 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>1300</v>
+        <v>2809.68</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>10 - ADM FINANCEIRO</t>
+          <t>13 - DES PRODUÇÃO</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -2218,22 +2210,22 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>2995</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -2243,20 +2235,16 @@
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>Idem</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr"/>
       <c r="K37" s="8" t="inlineStr"/>
       <c r="L37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>2809.68</v>
+        <v>4303.13</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
@@ -2265,7 +2253,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>8797 - DIAS BOLSA AUXILIO</t>
+          <t>8781 - DIAS NORMAIS</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2275,7 +2263,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>2910</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2285,12 +2273,12 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>2910</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>2526</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2298,22 +2286,26 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr"/>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>Conta certa; histórico sai como "DESC VALE REFEIÇÃO"</t>
+        </is>
+      </c>
       <c r="K38" s="8" t="inlineStr"/>
       <c r="L38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>4303.13</v>
+        <v>35</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>13 - DES PRODUÇÃO</t>
+          <t>14 - QUALIDADE</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>8781 - DIAS NORMAIS</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2323,7 +2315,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -2333,12 +2325,12 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2348,7 +2340,7 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>Conta certa; histórico sai como "DESC VALE REFEIÇÃO"</t>
+          <t>Invertido</t>
         </is>
       </c>
       <c r="K39" s="8" t="inlineStr"/>
@@ -2356,26 +2348,26 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>35</v>
+        <v>108.33</v>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>14 - QUALIDADE</t>
+          <t>16 - SD INFRAESTRUTURA</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
+          <t>8490 - BOLSA AUXILIO FERIAS</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Folha</t>
+          <t>Rescisão</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>3146</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -2385,22 +2377,22 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2526</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>Invertido</t>
+          <t>Rescisão de estágio do Lucas Meier (07/07) lançada em Ajuda de Custo do Suporte</t>
         </is>
       </c>
       <c r="K40" s="8" t="inlineStr"/>
@@ -2408,7 +2400,7 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>108.33</v>
+        <v>36.11</v>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
@@ -2417,7 +2409,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>8490 - BOLSA AUXILIO FERIAS</t>
+          <t>8496 - BOLSA AUXILIO 1/3 FERIAS</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2452,7 +2444,7 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de estágio do Lucas Meier (07/07) lançada em Ajuda de Custo do Suporte</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="K41" s="8" t="inlineStr"/>
@@ -2460,7 +2452,7 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>36.11</v>
+        <v>293.55</v>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
@@ -2469,7 +2461,7 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>8496 - BOLSA AUXILIO 1/3 FERIAS</t>
+          <t>8797 - DIAS BOLSA AUXILIO</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -2511,80 +2503,28 @@
       <c r="L42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
-        <v>293.55</v>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>16 - SD INFRAESTRUTURA</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>8797 - DIAS BOLSA AUXILIO</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>3146</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>2526</t>
-        </is>
-      </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J43" s="7" t="inlineStr">
-        <is>
-          <t>Idem</t>
-        </is>
-      </c>
-      <c r="K43" s="8" t="inlineStr"/>
-      <c r="L43" s="9" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="11">
-        <f>SUM(A5:A43)</f>
+      <c r="A43" s="10">
+        <f>SUM(A5:A42)</f>
         <v/>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="J44" s="13" t="inlineStr">
+      <c r="J43" s="12" t="inlineStr">
         <is>
           <t>Corrigidos:</t>
         </is>
       </c>
-      <c r="K44" s="12">
-        <f>COUNTIF(K5:K43,"Sim")&amp;" de "&amp;ROWS(K5:K43)</f>
+      <c r="K43" s="11">
+        <f>COUNTIF(K5:K42,"Sim")&amp;" de "&amp;ROWS(K5:K42)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K5:K43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>